<commit_message>
feat: master client bulk upload option added
</commit_message>
<xml_diff>
--- a/assets/templates/lead_upload_template.xlsx
+++ b/assets/templates/lead_upload_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lead Upload" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead Upload" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -152,6 +152,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>LeadCapture</author>
+  </authors>
+  <commentList>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Employee name or e-mail (as in Employee list). If filled, only that employee and admins can see this lead. Leave empty for no follow-up.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -441,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -459,6 +474,7 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="25" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -537,8 +553,14 @@
           <t>Created At (dd-MM-yyyy)</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Follow Up (Employee Name / Email)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: quick lead feature added
</commit_message>
<xml_diff>
--- a/assets/templates/lead_upload_template.xlsx
+++ b/assets/templates/lead_upload_template.xlsx
@@ -152,21 +152,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>LeadCapture</author>
-  </authors>
-  <commentList>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Employee name or e-mail (as in Employee list). If filled, only that employee and admins can see this lead. Leave empty for no follow-up.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -456,111 +441,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lead Name</t>
+          <t>Master Client (Company Name) *</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Contact Name (if new master client)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Contact Mobile (if new, 10 digits)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Name *</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Lead Email</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Lead Source</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Lead Category</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Lead Priority</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Lead Source *</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Category *</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Priority *</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status (default New)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Lead Value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Lead Status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Company Name</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Company Mobile</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Project Name</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Follow Up (Employee Name)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Project Description</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Created At (dd-MM-yyyy)</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Follow Up (Employee Name / Email)</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>